<commit_message>
chore: update rates (2026-09-15 08:41 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J114"/>
+  <dimension ref="A1:J117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4332,6 +4332,108 @@
         <v>3.62</v>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>3</v>
+      </c>
+      <c r="C115" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="D115" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="E115" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F115" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="G115" t="n">
+        <v>4.547</v>
+      </c>
+      <c r="H115" t="n">
+        <v>4.685</v>
+      </c>
+      <c r="I115" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="J115" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>3</v>
+      </c>
+      <c r="C116" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="D116" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="E116" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F116" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="G116" t="n">
+        <v>4.547</v>
+      </c>
+      <c r="H116" t="n">
+        <v>4.685</v>
+      </c>
+      <c r="I116" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="J116" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>3</v>
+      </c>
+      <c r="C117" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="D117" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="E117" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F117" t="n">
+        <v>4.138</v>
+      </c>
+      <c r="G117" t="n">
+        <v>4.558</v>
+      </c>
+      <c r="H117" t="n">
+        <v>4.686</v>
+      </c>
+      <c r="I117" t="n">
+        <v>4.021</v>
+      </c>
+      <c r="J117" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-09-16 07:01 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J117"/>
+  <dimension ref="A1:J118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4434,6 +4434,40 @@
         <v>3.62</v>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>3</v>
+      </c>
+      <c r="C118" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="D118" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="E118" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="F118" t="n">
+        <v>4.164</v>
+      </c>
+      <c r="G118" t="n">
+        <v>4.622</v>
+      </c>
+      <c r="H118" t="n">
+        <v>4.757</v>
+      </c>
+      <c r="I118" t="n">
+        <v>4.097</v>
+      </c>
+      <c r="J118" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-09-17 07:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J118"/>
+  <dimension ref="A1:J119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4468,6 +4468,40 @@
         <v>3.62</v>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>3</v>
+      </c>
+      <c r="C119" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D119" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E119" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="F119" t="n">
+        <v>4.186</v>
+      </c>
+      <c r="G119" t="n">
+        <v>4.593</v>
+      </c>
+      <c r="H119" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I119" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="J119" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-09-18 07:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J119"/>
+  <dimension ref="A1:J120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4502,6 +4502,40 @@
         <v>3.64</v>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>3</v>
+      </c>
+      <c r="C120" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D120" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E120" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F120" t="n">
+        <v>4.231</v>
+      </c>
+      <c r="G120" t="n">
+        <v>4.618</v>
+      </c>
+      <c r="H120" t="n">
+        <v>4.709</v>
+      </c>
+      <c r="I120" t="n">
+        <v>4.045</v>
+      </c>
+      <c r="J120" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: backfill rates (22 business days)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J120"/>
+  <dimension ref="A1:J121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4536,6 +4536,40 @@
         <v>3.62</v>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>3</v>
+      </c>
+      <c r="C121" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D121" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E121" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F121" t="n">
+        <v>4.258</v>
+      </c>
+      <c r="G121" t="n">
+        <v>4.617</v>
+      </c>
+      <c r="H121" t="n">
+        <v>4.691</v>
+      </c>
+      <c r="I121" t="n">
+        <v>4.027</v>
+      </c>
+      <c r="J121" t="n">
+        <v>3.85</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-09-22 07:32 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J121"/>
+  <dimension ref="A1:J124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4570,6 +4570,108 @@
         <v>3.85</v>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>3</v>
+      </c>
+      <c r="C122" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D122" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E122" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F122" t="n">
+        <v>4.258</v>
+      </c>
+      <c r="G122" t="n">
+        <v>4.617</v>
+      </c>
+      <c r="H122" t="n">
+        <v>4.691</v>
+      </c>
+      <c r="I122" t="n">
+        <v>4.027</v>
+      </c>
+      <c r="J122" t="n">
+        <v>3.85</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>3</v>
+      </c>
+      <c r="C123" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D123" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E123" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F123" t="n">
+        <v>4.258</v>
+      </c>
+      <c r="G123" t="n">
+        <v>4.617</v>
+      </c>
+      <c r="H123" t="n">
+        <v>4.691</v>
+      </c>
+      <c r="I123" t="n">
+        <v>4.027</v>
+      </c>
+      <c r="J123" t="n">
+        <v>3.85</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>3</v>
+      </c>
+      <c r="C124" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D124" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="E124" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F124" t="n">
+        <v>4.293</v>
+      </c>
+      <c r="G124" t="n">
+        <v>4.642</v>
+      </c>
+      <c r="H124" t="n">
+        <v>4.714</v>
+      </c>
+      <c r="I124" t="n">
+        <v>4.052</v>
+      </c>
+      <c r="J124" t="n">
+        <v>3.85</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-09-23 06:13 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J124"/>
+  <dimension ref="A1:J125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4672,6 +4672,40 @@
         <v>3.85</v>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>3</v>
+      </c>
+      <c r="C125" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="D125" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="E125" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F125" t="n">
+        <v>4.321</v>
+      </c>
+      <c r="G125" t="n">
+        <v>4.624</v>
+      </c>
+      <c r="H125" t="n">
+        <v>4.695</v>
+      </c>
+      <c r="I125" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="J125" t="n">
+        <v>3.85</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-09-24 06:26 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J125"/>
+  <dimension ref="A1:J126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4706,6 +4706,40 @@
         <v>3.85</v>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>3</v>
+      </c>
+      <c r="C126" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="D126" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="E126" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="F126" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="G126" t="n">
+        <v>4.604</v>
+      </c>
+      <c r="H126" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="I126" t="n">
+        <v>3.995</v>
+      </c>
+      <c r="J126" t="n">
+        <v>3.87</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-09-24 07:52 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -4712,9 +4712,7 @@
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="B126" t="n">
-        <v>3</v>
-      </c>
+      <c r="B126" t="inlineStr"/>
       <c r="C126" t="n">
         <v>3.21</v>
       </c>

</xml_diff>

<commit_message>
chore: update rates (2026-09-24 08:05 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -4712,7 +4712,9 @@
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr"/>
+      <c r="B126" t="n">
+        <v>3</v>
+      </c>
       <c r="C126" t="n">
         <v>3.21</v>
       </c>

</xml_diff>

<commit_message>
chore: update rates (2026-09-25 06:27 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J126"/>
+  <dimension ref="A1:J127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4740,6 +4740,40 @@
         <v>3.87</v>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>3</v>
+      </c>
+      <c r="C127" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="D127" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="E127" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="F127" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="G127" t="n">
+        <v>4.604</v>
+      </c>
+      <c r="H127" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="I127" t="n">
+        <v>3.995</v>
+      </c>
+      <c r="J127" t="n">
+        <v>3.87</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-09-29 07:57 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J128"/>
+  <dimension ref="A1:J131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4808,6 +4808,108 @@
         <v>3.88</v>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>3</v>
+      </c>
+      <c r="C129" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="D129" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="E129" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="F129" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="G129" t="n">
+        <v>4.604</v>
+      </c>
+      <c r="H129" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="I129" t="n">
+        <v>3.995</v>
+      </c>
+      <c r="J129" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>3</v>
+      </c>
+      <c r="C130" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="D130" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="E130" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="F130" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="G130" t="n">
+        <v>4.604</v>
+      </c>
+      <c r="H130" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="I130" t="n">
+        <v>3.995</v>
+      </c>
+      <c r="J130" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>3</v>
+      </c>
+      <c r="C131" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="D131" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="E131" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F131" t="n">
+        <v>4.405</v>
+      </c>
+      <c r="G131" t="n">
+        <v>4.697</v>
+      </c>
+      <c r="H131" t="n">
+        <v>4.777</v>
+      </c>
+      <c r="I131" t="n">
+        <v>4.111</v>
+      </c>
+      <c r="J131" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-09-30 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J131"/>
+  <dimension ref="A1:J132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4910,6 +4910,40 @@
         <v>3.9</v>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>3</v>
+      </c>
+      <c r="C132" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="D132" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="E132" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F132" t="n">
+        <v>4.416</v>
+      </c>
+      <c r="G132" t="n">
+        <v>4.666</v>
+      </c>
+      <c r="H132" t="n">
+        <v>4.738</v>
+      </c>
+      <c r="I132" t="n">
+        <v>4.072</v>
+      </c>
+      <c r="J132" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-01 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J132"/>
+  <dimension ref="A1:J133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4944,6 +4944,40 @@
         <v>3.9</v>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>3</v>
+      </c>
+      <c r="C133" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="D133" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E133" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="F133" t="n">
+        <v>4.385</v>
+      </c>
+      <c r="G133" t="n">
+        <v>4.619</v>
+      </c>
+      <c r="H133" t="n">
+        <v>4.682</v>
+      </c>
+      <c r="I133" t="n">
+        <v>4.015</v>
+      </c>
+      <c r="J133" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-02 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J133"/>
+  <dimension ref="A1:J134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4978,6 +4978,40 @@
         <v>3.88</v>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>3</v>
+      </c>
+      <c r="C134" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="D134" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="E134" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="F134" t="n">
+        <v>4.344</v>
+      </c>
+      <c r="G134" t="n">
+        <v>4.605</v>
+      </c>
+      <c r="H134" t="n">
+        <v>4.681</v>
+      </c>
+      <c r="I134" t="n">
+        <v>4.015</v>
+      </c>
+      <c r="J134" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-03 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J134"/>
+  <dimension ref="A1:J135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5012,6 +5012,40 @@
         <v>3.9</v>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>3</v>
+      </c>
+      <c r="C135" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="D135" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="E135" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F135" t="n">
+        <v>4.298</v>
+      </c>
+      <c r="G135" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="H135" t="n">
+        <v>4.595</v>
+      </c>
+      <c r="I135" t="n">
+        <v>3.927</v>
+      </c>
+      <c r="J135" t="n">
+        <v>3.87</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-06 08:59 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J135"/>
+  <dimension ref="A1:J138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5046,6 +5046,108 @@
         <v>3.87</v>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>3</v>
+      </c>
+      <c r="C136" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="D136" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="E136" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F136" t="n">
+        <v>4.298</v>
+      </c>
+      <c r="G136" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="H136" t="n">
+        <v>4.595</v>
+      </c>
+      <c r="I136" t="n">
+        <v>3.927</v>
+      </c>
+      <c r="J136" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>3</v>
+      </c>
+      <c r="C137" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="D137" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="E137" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F137" t="n">
+        <v>4.298</v>
+      </c>
+      <c r="G137" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="H137" t="n">
+        <v>4.595</v>
+      </c>
+      <c r="I137" t="n">
+        <v>3.927</v>
+      </c>
+      <c r="J137" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>3</v>
+      </c>
+      <c r="C138" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="D138" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="E138" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F138" t="n">
+        <v>4.298</v>
+      </c>
+      <c r="G138" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="H138" t="n">
+        <v>4.595</v>
+      </c>
+      <c r="I138" t="n">
+        <v>3.927</v>
+      </c>
+      <c r="J138" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-07 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J138"/>
+  <dimension ref="A1:J139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5148,6 +5148,40 @@
         <v>3.88</v>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>3</v>
+      </c>
+      <c r="C139" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="D139" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="E139" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F139" t="n">
+        <v>4.276</v>
+      </c>
+      <c r="G139" t="n">
+        <v>4.537</v>
+      </c>
+      <c r="H139" t="n">
+        <v>4.602</v>
+      </c>
+      <c r="I139" t="n">
+        <v>3.933</v>
+      </c>
+      <c r="J139" t="n">
+        <v>3.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-08 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J139"/>
+  <dimension ref="A1:J140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5182,6 +5182,40 @@
         <v>3.89</v>
       </c>
     </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>3</v>
+      </c>
+      <c r="C140" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="D140" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="E140" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F140" t="n">
+        <v>4.297</v>
+      </c>
+      <c r="G140" t="n">
+        <v>4.542</v>
+      </c>
+      <c r="H140" t="n">
+        <v>4.628</v>
+      </c>
+      <c r="I140" t="n">
+        <v>3.962</v>
+      </c>
+      <c r="J140" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-09 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J140"/>
+  <dimension ref="A1:J141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5216,6 +5216,40 @@
         <v>3.9</v>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>3</v>
+      </c>
+      <c r="C141" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="D141" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="E141" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="F141" t="n">
+        <v>4.298</v>
+      </c>
+      <c r="G141" t="n">
+        <v>4.566</v>
+      </c>
+      <c r="H141" t="n">
+        <v>4.663</v>
+      </c>
+      <c r="I141" t="n">
+        <v>3.997</v>
+      </c>
+      <c r="J141" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-10 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J141"/>
+  <dimension ref="A1:J142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5250,6 +5250,40 @@
         <v>3.88</v>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>3</v>
+      </c>
+      <c r="C142" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="D142" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="E142" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="F142" t="n">
+        <v>4.298</v>
+      </c>
+      <c r="G142" t="n">
+        <v>4.566</v>
+      </c>
+      <c r="H142" t="n">
+        <v>4.663</v>
+      </c>
+      <c r="I142" t="n">
+        <v>3.997</v>
+      </c>
+      <c r="J142" t="n">
+        <v>3.87</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-13 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J142"/>
+  <dimension ref="A1:J145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5284,6 +5284,108 @@
         <v>3.87</v>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>3</v>
+      </c>
+      <c r="C143" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="D143" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="E143" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="F143" t="n">
+        <v>4.298</v>
+      </c>
+      <c r="G143" t="n">
+        <v>4.566</v>
+      </c>
+      <c r="H143" t="n">
+        <v>4.663</v>
+      </c>
+      <c r="I143" t="n">
+        <v>3.997</v>
+      </c>
+      <c r="J143" t="n">
+        <v>3.87</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>3</v>
+      </c>
+      <c r="C144" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="D144" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="E144" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="F144" t="n">
+        <v>4.298</v>
+      </c>
+      <c r="G144" t="n">
+        <v>4.566</v>
+      </c>
+      <c r="H144" t="n">
+        <v>4.663</v>
+      </c>
+      <c r="I144" t="n">
+        <v>3.997</v>
+      </c>
+      <c r="J144" t="n">
+        <v>3.87</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>3</v>
+      </c>
+      <c r="C145" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="D145" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="E145" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="F145" t="n">
+        <v>4.276</v>
+      </c>
+      <c r="G145" t="n">
+        <v>4.514</v>
+      </c>
+      <c r="H145" t="n">
+        <v>4.588</v>
+      </c>
+      <c r="I145" t="n">
+        <v>3.918</v>
+      </c>
+      <c r="J145" t="n">
+        <v>3.87</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-14 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J145"/>
+  <dimension ref="A1:J146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5386,6 +5386,40 @@
         <v>3.87</v>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>3</v>
+      </c>
+      <c r="C146" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="D146" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="E146" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="F146" t="n">
+        <v>4.262</v>
+      </c>
+      <c r="G146" t="n">
+        <v>4.469</v>
+      </c>
+      <c r="H146" t="n">
+        <v>4.527</v>
+      </c>
+      <c r="I146" t="n">
+        <v>3.852</v>
+      </c>
+      <c r="J146" t="n">
+        <v>3.87</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-15 06:01 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J146"/>
+  <dimension ref="A1:J147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5420,6 +5420,40 @@
         <v>3.87</v>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>3</v>
+      </c>
+      <c r="C147" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="D147" t="n">
+        <v>3.61</v>
+      </c>
+      <c r="E147" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="F147" t="n">
+        <v>4.272</v>
+      </c>
+      <c r="G147" t="n">
+        <v>4.495</v>
+      </c>
+      <c r="H147" t="n">
+        <v>4.556</v>
+      </c>
+      <c r="I147" t="n">
+        <v>3.882</v>
+      </c>
+      <c r="J147" t="n">
+        <v>3.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-16 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J147"/>
+  <dimension ref="A1:J148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5454,6 +5454,40 @@
         <v>3.89</v>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>3</v>
+      </c>
+      <c r="C148" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="D148" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="E148" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F148" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="G148" t="n">
+        <v>4.484</v>
+      </c>
+      <c r="H148" t="n">
+        <v>4.546</v>
+      </c>
+      <c r="I148" t="n">
+        <v>3.872</v>
+      </c>
+      <c r="J148" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-17 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J148"/>
+  <dimension ref="A1:J149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5488,6 +5488,40 @@
         <v>3.88</v>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>3</v>
+      </c>
+      <c r="C149" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="D149" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="E149" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F149" t="n">
+        <v>4.267</v>
+      </c>
+      <c r="G149" t="n">
+        <v>4.452</v>
+      </c>
+      <c r="H149" t="n">
+        <v>4.512</v>
+      </c>
+      <c r="I149" t="n">
+        <v>3.835</v>
+      </c>
+      <c r="J149" t="n">
+        <v>3.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-20 06:01 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J149"/>
+  <dimension ref="A1:J152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5522,6 +5522,108 @@
         <v>3.89</v>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>3</v>
+      </c>
+      <c r="C150" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="D150" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="E150" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F150" t="n">
+        <v>4.267</v>
+      </c>
+      <c r="G150" t="n">
+        <v>4.452</v>
+      </c>
+      <c r="H150" t="n">
+        <v>4.512</v>
+      </c>
+      <c r="I150" t="n">
+        <v>3.835</v>
+      </c>
+      <c r="J150" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>3</v>
+      </c>
+      <c r="C151" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="D151" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="E151" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F151" t="n">
+        <v>4.267</v>
+      </c>
+      <c r="G151" t="n">
+        <v>4.452</v>
+      </c>
+      <c r="H151" t="n">
+        <v>4.512</v>
+      </c>
+      <c r="I151" t="n">
+        <v>3.835</v>
+      </c>
+      <c r="J151" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>3</v>
+      </c>
+      <c r="C152" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="D152" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="E152" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F152" t="n">
+        <v>4.292</v>
+      </c>
+      <c r="G152" t="n">
+        <v>4.478</v>
+      </c>
+      <c r="H152" t="n">
+        <v>4.553</v>
+      </c>
+      <c r="I152" t="n">
+        <v>3.877</v>
+      </c>
+      <c r="J152" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-21 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J152"/>
+  <dimension ref="A1:J153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5624,6 +5624,40 @@
         <v>3.88</v>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>3</v>
+      </c>
+      <c r="C153" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="D153" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E153" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F153" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="G153" t="n">
+        <v>4.438</v>
+      </c>
+      <c r="H153" t="n">
+        <v>4.512</v>
+      </c>
+      <c r="I153" t="n">
+        <v>3.835</v>
+      </c>
+      <c r="J153" t="n">
+        <v>3.87</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-22 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J153"/>
+  <dimension ref="A1:J154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5658,6 +5658,40 @@
         <v>3.87</v>
       </c>
     </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>3</v>
+      </c>
+      <c r="C154" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="D154" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="E154" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F154" t="n">
+        <v>4.282</v>
+      </c>
+      <c r="G154" t="n">
+        <v>4.418</v>
+      </c>
+      <c r="H154" t="n">
+        <v>4.492</v>
+      </c>
+      <c r="I154" t="n">
+        <v>3.811</v>
+      </c>
+      <c r="J154" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-23 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J154"/>
+  <dimension ref="A1:J155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5692,6 +5692,40 @@
         <v>3.88</v>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>3</v>
+      </c>
+      <c r="C155" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="D155" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="E155" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F155" t="n">
+        <v>4.286</v>
+      </c>
+      <c r="G155" t="n">
+        <v>4.439</v>
+      </c>
+      <c r="H155" t="n">
+        <v>4.516</v>
+      </c>
+      <c r="I155" t="n">
+        <v>3.837</v>
+      </c>
+      <c r="J155" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-24 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J155"/>
+  <dimension ref="A1:J156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5726,6 +5726,40 @@
         <v>3.88</v>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>3</v>
+      </c>
+      <c r="C156" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="D156" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="E156" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F156" t="n">
+        <v>4.267</v>
+      </c>
+      <c r="G156" t="n">
+        <v>4.426</v>
+      </c>
+      <c r="H156" t="n">
+        <v>4.489</v>
+      </c>
+      <c r="I156" t="n">
+        <v>3.809</v>
+      </c>
+      <c r="J156" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-27 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J156"/>
+  <dimension ref="A1:J159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5760,6 +5760,108 @@
         <v>3.9</v>
       </c>
     </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>3</v>
+      </c>
+      <c r="C157" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="D157" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="E157" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F157" t="n">
+        <v>4.267</v>
+      </c>
+      <c r="G157" t="n">
+        <v>4.426</v>
+      </c>
+      <c r="H157" t="n">
+        <v>4.489</v>
+      </c>
+      <c r="I157" t="n">
+        <v>3.809</v>
+      </c>
+      <c r="J157" t="n">
+        <v>3.92</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>3</v>
+      </c>
+      <c r="C158" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="D158" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="E158" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F158" t="n">
+        <v>4.267</v>
+      </c>
+      <c r="G158" t="n">
+        <v>4.426</v>
+      </c>
+      <c r="H158" t="n">
+        <v>4.489</v>
+      </c>
+      <c r="I158" t="n">
+        <v>3.809</v>
+      </c>
+      <c r="J158" t="n">
+        <v>3.92</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>3</v>
+      </c>
+      <c r="C159" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="D159" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="E159" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F159" t="n">
+        <v>4.255</v>
+      </c>
+      <c r="G159" t="n">
+        <v>4.407</v>
+      </c>
+      <c r="H159" t="n">
+        <v>4.468</v>
+      </c>
+      <c r="I159" t="n">
+        <v>3.787</v>
+      </c>
+      <c r="J159" t="n">
+        <v>3.92</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-28 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J159"/>
+  <dimension ref="A1:J160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5862,6 +5862,40 @@
         <v>3.92</v>
       </c>
     </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>3</v>
+      </c>
+      <c r="C160" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="D160" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="E160" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F160" t="n">
+        <v>4.245</v>
+      </c>
+      <c r="G160" t="n">
+        <v>4.379</v>
+      </c>
+      <c r="H160" t="n">
+        <v>4.445</v>
+      </c>
+      <c r="I160" t="n">
+        <v>3.762</v>
+      </c>
+      <c r="J160" t="n">
+        <v>3.93</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-29 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J160"/>
+  <dimension ref="A1:J161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5896,6 +5896,40 @@
         <v>3.93</v>
       </c>
     </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>3</v>
+      </c>
+      <c r="C161" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="D161" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="E161" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F161" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="G161" t="n">
+        <v>4.414</v>
+      </c>
+      <c r="H161" t="n">
+        <v>4.484</v>
+      </c>
+      <c r="I161" t="n">
+        <v>3.802</v>
+      </c>
+      <c r="J161" t="n">
+        <v>3.95</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-30 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J161"/>
+  <dimension ref="A1:J162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5930,6 +5930,40 @@
         <v>3.95</v>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>3</v>
+      </c>
+      <c r="C162" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="D162" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="E162" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F162" t="n">
+        <v>4.236</v>
+      </c>
+      <c r="G162" t="n">
+        <v>4.378</v>
+      </c>
+      <c r="H162" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="I162" t="n">
+        <v>3.755</v>
+      </c>
+      <c r="J162" t="n">
+        <v>3.94</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update rates (2026-10-31 06:00 KST)
</commit_message>
<xml_diff>
--- a/docs/data/history.xlsx
+++ b/docs/data/history.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J162"/>
+  <dimension ref="A1:J163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5964,6 +5964,40 @@
         <v>3.94</v>
       </c>
     </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>3</v>
+      </c>
+      <c r="C163" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="D163" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="E163" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="F163" t="n">
+        <v>4.217</v>
+      </c>
+      <c r="G163" t="n">
+        <v>4.343</v>
+      </c>
+      <c r="H163" t="n">
+        <v>4.394</v>
+      </c>
+      <c r="I163" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="J163" t="n">
+        <v>3.94</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>